<commit_message>
Final code review and cleanup for IT delivery
Services (services/src/):
- Fix gap filling bug in file_research_subagent.py (chunk_id key)
- Update all agents with refined prompts and error handling
- Improve cascading retrieval architecture (metadata + file research)
- Standardize docstrings per project documentation standards
- Add linting config (.flake8, .pylintrc)

Database Config (db_config/):
- Update registry schema with new research config fields
- Consolidate prompt backups (remove deprecated global prompts)
- Add metadata_context_fields to all database registries

Doc Refresh (doc_refresh/):
- Standardize utilities (env_config, prompt_loader, fiscal_context)
- Align with services module patterns

Cleanup:
- Remove obsolete notes/ folder (implementation plans, old documentation)
- Remove deprecated testing scripts and data exports
- Remove unused migration files

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testing/agent_tests/input/test_cases.xlsx
+++ b/testing/agent_tests/input/test_cases.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Router" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Clarifier" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Planner" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DirectResponse" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summarizer" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Router" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clarifier" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planner" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DirectResponse" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summarizer" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1827,6 +1827,276 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>RT051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Thanks plus new question</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "Tell me about IFRS 16"}, {"role": "assistant", "content": "IFRS 16 covers lease accounting requirements."}, {"role": "user", "content": "Thanks! What about goodwill impairment testing?"}]</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>database_research</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Mixed thanks with new question - should route to research</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>RT052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Great now tell me</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "What is hedge accounting?"}, {"role": "assistant", "content": "Hedge accounting aligns accounting with risk management strategies."}, {"role": "user", "content": "Great, now tell me about deferred tax accounting."}]</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>database_research</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Acknowledgment followed by new topic</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>RT053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>That helps but also</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "Explain IFRS 9"}, {"role": "assistant", "content": "IFRS 9 is the standard for financial instruments."}, {"role": "user", "content": "That helps, but can you also explain the ECL model in detail from our policy?"}]</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>database_research</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Appreciation with request for policy detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>RT054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Understood now different</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "What is revenue recognition?"}, {"role": "assistant", "content": "Revenue recognition determines when to record revenue."}, {"role": "user", "content": "Understood. Now, what are the PAR approval requirements?"}]</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>database_research</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Acknowledgment then completely different topic</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>RT055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Perfect one more thing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "How do we account for leases?"}, {"role": "assistant", "content": "Under IFRS 16, leases are recognized on balance sheet."}, {"role": "user", "content": "Perfect! One more thing - what's our policy on related party transactions?"}]</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>database_research</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Praise followed by new policy question</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>RT056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Tell me more policy detail</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "What is IFRS 15?"}, {"role": "assistant", "content": "IFRS 15 is the revenue recognition standard."}, {"role": "user", "content": "Tell me more about the five-step model in detail from our policy manual."}]</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>database_research</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Request for policy manual details requires research</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>RT057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Expand specific requirements</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "Brief overview of hedge accounting"}, {"role": "assistant", "content": "Hedge accounting aligns accounting treatment with risk management."}, {"role": "user", "content": "Can you expand on the specific hedge effectiveness testing requirements in RBC policy?"}]</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>database_research</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Request for specific policy details</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>RT058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>What does policy say</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "Give me an overview of impairment"}, {"role": "assistant", "content": "Impairment reduces asset values when recoverable amount is less than carrying amount."}, {"role": "user", "content": "What does our policy manual specifically say about impairment indicators?"}]</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>database_research</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Request for policy specifics requires lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>RT059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Simpler explanation direct</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "Explain IFRS 9 classification"}, {"role": "assistant", "content": "IFRS 9 classifies financial assets based on business model and contractual cash flow characteristics into amortized cost, FVOCI, or FVTPL."}, {"role": "user", "content": "Can you explain that in simpler terms?"}]</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>direct_response</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Request for simpler explanation of existing content</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>RT060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Give me an example direct</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "What is a performance obligation?"}, {"role": "assistant", "content": "A performance obligation is a promise to transfer a distinct good or service to a customer."}, {"role": "user", "content": "Can you give me an example?"}]</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>direct_response</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Request for example can use general knowledge</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1838,7 +2108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2423,22 +2693,22 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Derecognition financial assets</t>
+          <t>Find all documents topic</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What are the criteria for derecognition of financial assets?"}]</t>
+          <t>[{"role": "user", "content": "What documents do we have about revenue recognition?"}]</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>proceed_with_research</t>
+          <t>request_deep_research_approval</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Derecognition criteria</t>
+          <t>Discovery query - needs comprehensive search</t>
         </is>
       </c>
     </row>
@@ -2450,22 +2720,22 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Lease incentives treatment</t>
+          <t>List all policies</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "How are lease incentives accounted for by the lessee?"}]</t>
+          <t>[{"role": "user", "content": "List all our policies related to leasing."}]</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>proceed_with_research</t>
+          <t>request_deep_research_approval</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Lease incentives</t>
+          <t>Comprehensive listing request</t>
         </is>
       </c>
     </row>
@@ -2477,22 +2747,22 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Principal vs agent</t>
+          <t>Give me everything</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "How do you determine if an entity is acting as principal or agent for revenue recognition?"}]</t>
+          <t>[{"role": "user", "content": "Give me everything we have on IFRS 9."}]</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>proceed_with_research</t>
+          <t>request_deep_research_approval</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Principal vs agent</t>
+          <t>Comprehensive search request</t>
         </is>
       </c>
     </row>
@@ -2504,22 +2774,22 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Impairment stages</t>
+          <t>All guidance on topic</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What are the three stages of impairment under the ECL model?"}]</t>
+          <t>[{"role": "user", "content": "Show me all the guidance on hedge accounting."}]</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>proceed_with_research</t>
+          <t>request_deep_research_approval</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>ECL stages</t>
+          <t>Request for all materials</t>
         </is>
       </c>
     </row>
@@ -2531,22 +2801,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Sale and leaseback</t>
+          <t>Comprehensive overview</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "How should a sale and leaseback transaction be accounted for under IFRS 16?"}]</t>
+          <t>[{"role": "user", "content": "I need a comprehensive overview of all our financial instruments policies."}]</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>proceed_with_research</t>
+          <t>request_deep_research_approval</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Sale leaseback</t>
+          <t>Comprehensive request</t>
         </is>
       </c>
     </row>
@@ -2558,22 +2828,22 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Vague accounting question</t>
+          <t>What references exist</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "Tell me about accounting"}]</t>
+          <t>[{"role": "user", "content": "What references exist in our documentation for impairment?"}]</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ask_clarification</t>
+          <t>request_deep_research_approval</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Too broad</t>
+          <t>Discovery of all references</t>
         </is>
       </c>
     </row>
@@ -2585,22 +2855,22 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Just leases</t>
+          <t>Search entire database</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "Leases"}]</t>
+          <t>[{"role": "user", "content": "Search the entire database for mentions of cryptocurrency."}]</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>ask_clarification</t>
+          <t>request_deep_research_approval</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Single word, no context</t>
+          <t>Explicit full database search</t>
         </is>
       </c>
     </row>
@@ -2612,22 +2882,22 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Help with something</t>
+          <t>Every document mentioning</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "I need help with something"}]</t>
+          <t>[{"role": "user", "content": "Find every document that mentions ESG reporting."}]</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>ask_clarification</t>
+          <t>request_deep_research_approval</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Unspecified need</t>
+          <t>Request for all documents</t>
         </is>
       </c>
     </row>
@@ -2639,22 +2909,22 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>How does it work</t>
+          <t>Inventory of policies</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "How does it work?"}]</t>
+          <t>[{"role": "user", "content": "Can you provide an inventory of all accounting policies we have?"}]</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>ask_clarification</t>
+          <t>request_deep_research_approval</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Missing subject</t>
+          <t>Full inventory request</t>
         </is>
       </c>
     </row>
@@ -2666,22 +2936,22 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Vague standards question</t>
+          <t>Complete coverage</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What are the standards?"}]</t>
+          <t>[{"role": "user", "content": "I want complete coverage of all consolidation-related guidance."}]</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>ask_clarification</t>
+          <t>request_deep_research_approval</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Which standards?</t>
+          <t>Complete coverage request</t>
         </is>
       </c>
     </row>
@@ -2693,12 +2963,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>General policy question</t>
+          <t>Vague accounting question</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What's the policy?"}]</t>
+          <t>[{"role": "user", "content": "Tell me about accounting"}]</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2708,7 +2978,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Which policy?</t>
+          <t>Too vague - which area of accounting?</t>
         </is>
       </c>
     </row>
@@ -2720,12 +2990,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous treatment</t>
+          <t>Just leases</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What's the treatment?"}]</t>
+          <t>[{"role": "user", "content": "Leases"}]</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2735,7 +3005,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Treatment of what?</t>
+          <t>Single word - what aspect of leases?</t>
         </is>
       </c>
     </row>
@@ -2747,12 +3017,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Vague guidance request</t>
+          <t>Help with something</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "I need guidance"}]</t>
+          <t>[{"role": "user", "content": "I need help with something"}]</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2762,7 +3032,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Guidance on what?</t>
+          <t>Too vague - help with what?</t>
         </is>
       </c>
     </row>
@@ -2774,12 +3044,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Something about revenue</t>
+          <t>How does it work</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "Something about revenue"}]</t>
+          <t>[{"role": "user", "content": "How does it work?"}]</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2789,7 +3059,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Vague revenue question</t>
+          <t>Missing subject - how does WHAT work?</t>
         </is>
       </c>
     </row>
@@ -2801,12 +3071,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Generic IFRS question</t>
+          <t>Vague standards question</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What about IFRS?"}]</t>
+          <t>[{"role": "user", "content": "What are the standards?"}]</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2816,7 +3086,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Which IFRS standard?</t>
+          <t>Too vague - which standards for what?</t>
         </is>
       </c>
     </row>
@@ -2828,12 +3098,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Incomplete question</t>
+          <t>General policy question</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "How do I..."}]</t>
+          <t>[{"role": "user", "content": "What's the policy?"}]</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2843,7 +3113,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Incomplete</t>
+          <t>Which policy?</t>
         </is>
       </c>
     </row>
@@ -2855,12 +3125,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Vague comparison</t>
+          <t>Ambiguous treatment</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "Compare them"}]</t>
+          <t>[{"role": "user", "content": "What's the treatment?"}]</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2870,7 +3140,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Compare what?</t>
+          <t>Treatment of what?</t>
         </is>
       </c>
     </row>
@@ -2882,12 +3152,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Generic rules question</t>
+          <t>Vague guidance request</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What are the rules?"}]</t>
+          <t>[{"role": "user", "content": "I need guidance"}]</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2897,7 +3167,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Rules for what?</t>
+          <t>Guidance on what?</t>
         </is>
       </c>
     </row>
@@ -2909,12 +3179,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous measurement</t>
+          <t>Something about revenue</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "How is it measured?"}]</t>
+          <t>[{"role": "user", "content": "Something about revenue"}]</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2924,7 +3194,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>What is measured?</t>
+          <t>Vague revenue question</t>
         </is>
       </c>
     </row>
@@ -2936,12 +3206,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Vague asset question</t>
+          <t>Generic IFRS question</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "Tell me about assets"}]</t>
+          <t>[{"role": "user", "content": "What about IFRS?"}]</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2951,7 +3221,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Which type of assets?</t>
+          <t>Which IFRS standard?</t>
         </is>
       </c>
     </row>
@@ -2963,12 +3233,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Generic disclosure question</t>
+          <t>Incomplete question</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What disclosures are needed?"}]</t>
+          <t>[{"role": "user", "content": "How do I..."}]</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2978,7 +3248,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Disclosures for what?</t>
+          <t>Incomplete</t>
         </is>
       </c>
     </row>
@@ -2990,12 +3260,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous timing</t>
+          <t>Vague comparison</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "When do we recognize it?"}]</t>
+          <t>[{"role": "user", "content": "Compare them"}]</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -3005,7 +3275,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Recognize what?</t>
+          <t>Compare what?</t>
         </is>
       </c>
     </row>
@@ -3017,12 +3287,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Vague impairment</t>
+          <t>Generic rules question</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "Impairment rules"}]</t>
+          <t>[{"role": "user", "content": "What are the rules?"}]</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -3032,7 +3302,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Impairment of what?</t>
+          <t>Rules for what?</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3314,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Generic classification</t>
+          <t>Ambiguous measurement</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "How is it classified?"}]</t>
+          <t>[{"role": "user", "content": "How is it measured?"}]</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -3059,7 +3329,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Classify what?</t>
+          <t>What is measured?</t>
         </is>
       </c>
     </row>
@@ -3071,12 +3341,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous contract</t>
+          <t>Vague asset question</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What about the contract?"}]</t>
+          <t>[{"role": "user", "content": "Tell me about assets"}]</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -3086,7 +3356,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Which contract aspect?</t>
+          <t>Which type of assets?</t>
         </is>
       </c>
     </row>
@@ -3098,12 +3368,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Vague modification</t>
+          <t>Generic disclosure question</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "Modifications"}]</t>
+          <t>[{"role": "user", "content": "What disclosures are needed?"}]</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -3113,7 +3383,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Modifications to what?</t>
+          <t>Disclosures for what?</t>
         </is>
       </c>
     </row>
@@ -3125,12 +3395,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Generic criteria</t>
+          <t>Ambiguous timing</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What are the criteria?"}]</t>
+          <t>[{"role": "user", "content": "When do we recognize it?"}]</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -3140,7 +3410,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Criteria for what?</t>
+          <t>Recognize what?</t>
         </is>
       </c>
     </row>
@@ -3152,12 +3422,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous calculation</t>
+          <t>Vague impairment</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "How do you calculate that?"}]</t>
+          <t>[{"role": "user", "content": "Impairment rules"}]</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -3167,7 +3437,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Calculate what?</t>
+          <t>Impairment of what?</t>
         </is>
       </c>
     </row>
@@ -3179,12 +3449,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Vague requirements</t>
+          <t>Generic classification</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>[{"role": "user", "content": "What are the requirements?"}]</t>
+          <t>[{"role": "user", "content": "How is it classified?"}]</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -3194,7 +3464,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Requirements for what?</t>
+          <t>Classify what?</t>
         </is>
       </c>
     </row>
@@ -3206,22 +3476,292 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
+          <t>Ambiguous contract</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "What about the contract?"}]</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>ask_clarification</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Which contract aspect?</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CL051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Vague modification</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "Modifications"}]</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ask_clarification</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Modifications to what?</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CL052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Generic criteria</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "What are the criteria?"}]</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ask_clarification</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Criteria for what?</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>CL053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Ambiguous calculation</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "How do you calculate that?"}]</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ask_clarification</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Calculate what?</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CL054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Vague requirements</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "What are the requirements?"}]</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ask_clarification</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Requirements for what?</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>CL055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>Generic obligation</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>[{"role": "user", "content": "What's the obligation?"}]</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>ask_clarification</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>Which obligation?</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CL056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Specific IFRS 17 question</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "What are the general measurement requirements under IFRS 17?"}]</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>proceed_with_research</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Clear IFRS 17 question</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CL057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Business combination goodwill</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "How is goodwill calculated in a business combination under IFRS 3?"}]</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>proceed_with_research</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Clear business combination question</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>CL058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Foreign currency translation</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "What are the requirements for translating foreign currency transactions under IAS 21?"}]</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>proceed_with_research</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Clear IAS 21 question</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>CL059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Related party identification</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "How do you identify related parties under IAS 24?"}]</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>proceed_with_research</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Clear IAS 24 question</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>CL060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Provisions recognition criteria</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>[{"role": "user", "content": "What are the recognition criteria for provisions under IAS 37?"}]</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>proceed_with_research</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Clear IAS 37 question</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4911,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>internal_capm</t>
+          <t>internal_capm,external_ey</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -4393,12 +4933,12 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Compare RBC revenue policy with IASB standards and EY interpretations</t>
+          <t>Compare RBC revenue recognition accounting policy with IASB IFRS 15 standards and EY interpretations</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>internal_capm</t>
+          <t>internal_capm,external_iasb,external_ey</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -4425,7 +4965,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>internal_capm</t>
+          <t>internal_capm,external_iasb,external_ey</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -4452,7 +4992,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>internal_capm</t>
+          <t>internal_capm,external_ey</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -4479,7 +5019,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>internal_capm</t>
+          <t>internal_capm,internal_memos,internal_wiki</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -4506,7 +5046,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>internal_capm</t>
+          <t>internal_capm,internal_memos,internal_cheatsheets</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -4533,7 +5073,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>external_ey</t>
+          <t>external_ey,external_iasb</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -4560,7 +5100,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>internal_capm</t>
+          <t>internal_capm,internal_memos</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -4587,7 +5127,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>internal_capm</t>
+          <t>internal_ext_reporting_and_disclosure,external_iasb,external_ey</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -4614,7 +5154,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>internal_capm</t>
+          <t>external_iasb,external_ey</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">

</xml_diff>